<commit_message>
release: curated nRF52840 system with Rev J KiCad and firmware history
</commit_message>
<xml_diff>
--- a/mau/ARS_du_lieu_thu.xlsx
+++ b/mau/ARS_du_lieu_thu.xlsx
@@ -536,12 +536,6 @@
           <t>SMTP</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>B</t>
@@ -590,12 +584,6 @@
           <t>Không đảm bảo</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>B</t>
@@ -644,12 +632,6 @@
           <t>Giữ kết nối</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>B</t>
@@ -693,13 +675,6 @@
           <t>5 GHz</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
           <t>B</t>
@@ -738,14 +713,6 @@
           <t>Không</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>B</t>
@@ -799,11 +766,6 @@
           <t>NE555</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>C</t>
@@ -847,13 +809,6 @@
           <t>Chân ADC</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
           <t>B</t>
@@ -907,12 +862,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>23134001</t>
+          <t>DEMO001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Lê Văn Giang</t>
+          <t>Học sinh mẫu 01</t>
         </is>
       </c>
     </row>
@@ -922,12 +877,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>23134002</t>
+          <t>DEMO002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Trần Ngọc Thảo</t>
+          <t>Học sinh mẫu 02</t>
         </is>
       </c>
     </row>
@@ -937,12 +892,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>23134003</t>
+          <t>DEMO003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Bùi Ngọc Phúc</t>
+          <t>Học sinh mẫu 03</t>
         </is>
       </c>
     </row>
@@ -952,12 +907,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>23134004</t>
+          <t>DEMO004</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Đặng Thị Bình</t>
+          <t>Học sinh mẫu 04</t>
         </is>
       </c>
     </row>
@@ -967,12 +922,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>23134005</t>
+          <t>DEMO005</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Bùi Văn Vy</t>
+          <t>Học sinh mẫu 05</t>
         </is>
       </c>
     </row>
@@ -982,12 +937,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>23134006</t>
+          <t>DEMO006</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Đặng Ngọc Nam</t>
+          <t>Học sinh mẫu 06</t>
         </is>
       </c>
     </row>
@@ -997,12 +952,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>23134007</t>
+          <t>DEMO007</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Nguyễn Ngọc Giang</t>
+          <t>Học sinh mẫu 07</t>
         </is>
       </c>
     </row>
@@ -1012,12 +967,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>23134008</t>
+          <t>DEMO008</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Phạm Văn Vy</t>
+          <t>Học sinh mẫu 08</t>
         </is>
       </c>
     </row>
@@ -1027,12 +982,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>23134009</t>
+          <t>DEMO009</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Võ Văn An</t>
+          <t>Học sinh mẫu 09</t>
         </is>
       </c>
     </row>
@@ -1042,12 +997,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>23134010</t>
+          <t>DEMO010</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Nguyễn Văn Vy</t>
+          <t>Học sinh mẫu 10</t>
         </is>
       </c>
     </row>
@@ -1057,12 +1012,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>23134011</t>
+          <t>DEMO011</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Đặng Thị Khánh</t>
+          <t>Học sinh mẫu 11</t>
         </is>
       </c>
     </row>
@@ -1072,12 +1027,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>23134012</t>
+          <t>DEMO012</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Nguyễn Thị Thảo</t>
+          <t>Học sinh mẫu 12</t>
         </is>
       </c>
     </row>
@@ -1087,12 +1042,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>23134013</t>
+          <t>DEMO013</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Bùi Ngọc Minh</t>
+          <t>Học sinh mẫu 13</t>
         </is>
       </c>
     </row>
@@ -1102,12 +1057,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>23134014</t>
+          <t>DEMO014</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Phạm Minh Dũng</t>
+          <t>Học sinh mẫu 14</t>
         </is>
       </c>
     </row>
@@ -1117,12 +1072,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>23134015</t>
+          <t>DEMO015</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Phạm Ngọc Giang</t>
+          <t>Học sinh mẫu 15</t>
         </is>
       </c>
     </row>
@@ -1132,12 +1087,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>23134016</t>
+          <t>DEMO016</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Nguyễn Ngọc Tùng</t>
+          <t>Học sinh mẫu 16</t>
         </is>
       </c>
     </row>
@@ -1147,12 +1102,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>23134017</t>
+          <t>DEMO017</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Trần Thị Phúc</t>
+          <t>Học sinh mẫu 17</t>
         </is>
       </c>
     </row>
@@ -1162,12 +1117,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>23134018</t>
+          <t>DEMO018</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Hoàng Văn Quân</t>
+          <t>Học sinh mẫu 18</t>
         </is>
       </c>
     </row>
@@ -1177,12 +1132,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>23134019</t>
+          <t>DEMO019</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Võ Ngọc Minh</t>
+          <t>Học sinh mẫu 19</t>
         </is>
       </c>
     </row>
@@ -1192,12 +1147,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>23134020</t>
+          <t>DEMO020</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Phạm Minh Giang</t>
+          <t>Học sinh mẫu 20</t>
         </is>
       </c>
     </row>
@@ -1207,12 +1162,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>23134021</t>
+          <t>DEMO021</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Bùi Ngọc Nam</t>
+          <t>Học sinh mẫu 21</t>
         </is>
       </c>
     </row>
@@ -1222,12 +1177,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>23134022</t>
+          <t>DEMO022</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Nguyễn Ngọc Dũng</t>
+          <t>Học sinh mẫu 22</t>
         </is>
       </c>
     </row>
@@ -1237,12 +1192,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>23134023</t>
+          <t>DEMO023</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Đặng Ngọc Phúc</t>
+          <t>Học sinh mẫu 23</t>
         </is>
       </c>
     </row>
@@ -1252,12 +1207,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>23134024</t>
+          <t>DEMO024</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Lê Minh Minh</t>
+          <t>Học sinh mẫu 24</t>
         </is>
       </c>
     </row>
@@ -1267,12 +1222,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>23134025</t>
+          <t>DEMO025</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Võ Văn Linh</t>
+          <t>Học sinh mẫu 25</t>
         </is>
       </c>
     </row>
@@ -1282,12 +1237,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>23134026</t>
+          <t>DEMO026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Trần Thị Minh</t>
+          <t>Học sinh mẫu 26</t>
         </is>
       </c>
     </row>
@@ -1297,12 +1252,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>23134027</t>
+          <t>DEMO027</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Đặng Minh Linh</t>
+          <t>Học sinh mẫu 27</t>
         </is>
       </c>
     </row>
@@ -1312,12 +1267,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>23134028</t>
+          <t>DEMO028</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Nguyễn Ngọc An</t>
+          <t>Học sinh mẫu 28</t>
         </is>
       </c>
     </row>
@@ -1327,12 +1282,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>23134029</t>
+          <t>DEMO029</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Hoàng Ngọc Phúc</t>
+          <t>Học sinh mẫu 29</t>
         </is>
       </c>
     </row>
@@ -1342,12 +1297,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>23134030</t>
+          <t>DEMO030</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Lê Thị Minh</t>
+          <t>Học sinh mẫu 30</t>
         </is>
       </c>
     </row>
@@ -1357,12 +1312,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>23134031</t>
+          <t>DEMO031</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Phạm Văn Thảo</t>
+          <t>Học sinh mẫu 31</t>
         </is>
       </c>
     </row>
@@ -1372,12 +1327,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>23134032</t>
+          <t>DEMO032</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Phạm Thị Khánh</t>
+          <t>Học sinh mẫu 32</t>
         </is>
       </c>
     </row>
@@ -1387,12 +1342,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>23134033</t>
+          <t>DEMO033</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Võ Minh Linh</t>
+          <t>Học sinh mẫu 33</t>
         </is>
       </c>
     </row>
@@ -1402,12 +1357,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>23134034</t>
+          <t>DEMO034</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Hoàng Văn Khánh</t>
+          <t>Học sinh mẫu 34</t>
         </is>
       </c>
     </row>
@@ -1417,12 +1372,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>23134035</t>
+          <t>DEMO035</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Lê Thị Khánh</t>
+          <t>Học sinh mẫu 35</t>
         </is>
       </c>
     </row>
@@ -1432,12 +1387,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>23134036</t>
+          <t>DEMO036</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Nguyễn Ngọc Tùng</t>
+          <t>Học sinh mẫu 36</t>
         </is>
       </c>
     </row>
@@ -1447,12 +1402,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>23134037</t>
+          <t>DEMO037</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Võ Thị Minh</t>
+          <t>Học sinh mẫu 37</t>
         </is>
       </c>
     </row>
@@ -1462,12 +1417,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>23134038</t>
+          <t>DEMO038</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Đặng Ngọc Tùng</t>
+          <t>Học sinh mẫu 38</t>
         </is>
       </c>
     </row>
@@ -1477,12 +1432,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>23134039</t>
+          <t>DEMO039</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Võ Ngọc Hà</t>
+          <t>Học sinh mẫu 39</t>
         </is>
       </c>
     </row>
@@ -1492,12 +1447,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>23134040</t>
+          <t>DEMO040</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Nguyễn Minh Linh</t>
+          <t>Học sinh mẫu 40</t>
         </is>
       </c>
     </row>

</xml_diff>